<commit_message>
Refactor notebook and paper builders for clarity and accuracy in text analysis
- Updated conclusion and limitations sections in notebook to reflect new validation results and methodology.
- Enhanced the robustness analysis in the paper builder, clarifying the use of EGARCH-X and its implications.
- Improved the description of manual validation processes and results, emphasizing the distinction between initial dictionaries and supervised models.
- Adjusted formatting and structure for better readability and consistency across sections.
- Added detailed explanations for statistical methods and their relevance to the findings.
</commit_message>
<xml_diff>
--- a/paper/引用一致性审计.xlsx
+++ b/paper/引用一致性审计.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="references" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,293 +413,143 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>reference_no</t>
+          <t>citation</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>citation</t>
+          <t>appears_in_body</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>in_reference_list</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>verification_url</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>doi_or_id</t>
+          <t>reference</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>姜富伟、胡逸驰、黄楠（2021）：《央行货币政策报告文本信息、宏观经济与股票市场》，《金融研究》第6期。</t>
-        </is>
-      </c>
-      <c r="C2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.jryj.org.cn/CN/abstract/abstract897.shtml</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>姜富伟、胡逸驰、黄楠：《央行货币政策报告文本信息、宏观经济与股票市场》，《金融研究》，2021年第6期。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>董青马、张皓越、马剑文、尚玉皇（2024）：《央行沟通与资产价格——识别“潜在”未预期货币政策信息》，《金融研究》2024年第6期。</t>
-        </is>
-      </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.jryj.org.cn/CN/abstract/abstract1334.shtml</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>董青马、张皓越、马剑文、尚玉皇：《央行沟通与资产价格：识别“潜在”未预期货币政策信息》，《金融研究》，2024年第6期。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>尚玉皇、刘华、申峰（2025）：《预期的博弈：央行沟通与国债收益率曲线》，《金融研究》2025年第9期。</t>
-        </is>
-      </c>
-      <c r="C4" t="b">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.jryj.org.cn/CN/abstract/abstract1520.shtml</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>尚玉皇、刘华、申峰：《预期的博弈：央行沟通与国债收益率曲线》，《金融研究》，2025年第9期。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>McMahon, M., Schipke, A., &amp; Li, X. (2018). China's Monetary Policy Communication: Frameworks, Impact, and Recommendations. IMF Working Paper 2018/244.</t>
-        </is>
-      </c>
-      <c r="C5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.imf.org/en/publications/wp/issues/2018/11/17/chinas-monetary-policy-communication-frameworks-impact-and-recommendations-46375</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>10.5089/9781484385647.001</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Du Z., Huang A. G., Wermers R. and Wu W. Language and Domain Specificity: A Chinese Financial Sentiment Dictionary. Review of Finance, 2022, 26(3): 673-719.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Blinder, A. S., Ehrmann, M., Fratzscher, M., de Haan, J., &amp; Jansen, D. (2008). Central Bank Communication and Monetary Policy: A Survey of Theory and Evidence. Journal of Economic Literature, 46(4), 910-945.</t>
-        </is>
-      </c>
-      <c r="C6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.aeaweb.org/articles?id=10.1257%2Fjel.46.4.910</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>10.1257/jel.46.4.910</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>[5]</t>
+        </is>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Gurkaynak R. S., Sack B. and Swanson E. Do Actions Speak Louder Than Words? The Response of Asset Prices to Monetary Policy Actions and Statements. International Journal of Central Banking, 2005, 1(1): 55-93.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Gurkaynak, R. S., Sack, B., &amp; Swanson, E. T. (2005). Do Actions Speak Louder Than Words? The Response of Asset Prices to Monetary Policy Actions and Statements. International Journal of Central Banking, 1(1), 55-93.</t>
-        </is>
-      </c>
-      <c r="C7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://www.ijcb.org/journal/v1n1/do-actions-speak-louder-words-response-asset-prices-monetary-policy-actions-and</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>[6]</t>
+        </is>
+      </c>
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tetlock P. C. Giving Content to Investor Sentiment: The Role of Media in the Stock Market. Journal of Finance, 2007, 62(3): 1139-1168.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Kuttner, K. N. (2001). Monetary Policy Surprises and Interest Rates: Evidence from the Fed Funds Futures Market. Journal of Monetary Economics, 47(3), 523-544.</t>
-        </is>
-      </c>
-      <c r="C8" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://ideas.repec.org/a/eee/moneco/v47y2001i3p523-544.html</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>10.1016/S0304-3932(01)00055-1</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>[7]</t>
+        </is>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Nelson D. B. Conditional Heteroskedasticity in Asset Returns: A New Approach. Econometrica, 1991, 59(2): 347-370.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Hansen, S., &amp; McMahon, M. (2016). Shocking Language: Understanding the Macroeconomic Effects of Central Bank Communication. Journal of International Economics, 99, S114-S133.</t>
-        </is>
-      </c>
-      <c r="C9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://wrap.warwick.ac.uk/id/eprint/85615/</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>10.1016/j.jinteco.2015.12.008</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Nakamura, E., &amp; Steinsson, J. (2018). High-Frequency Identification of Monetary Non-Neutrality: The Information Effect. Quarterly Journal of Economics, 133(3), 1283-1330.</t>
-        </is>
-      </c>
-      <c r="C10" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://academic.oup.com/qje/article-abstract/133/3/1283/4828341</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>10.1093/qje/qjy004</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Jarocinski, M., &amp; Karadi, P. (2020). Deconstructing Monetary Policy Surprises: The Role of Information Shocks. American Economic Journal: Macroeconomics, 12(2), 1-43.</t>
-        </is>
-      </c>
-      <c r="C11" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://www.aeaweb.org/articles?id=10.1257%2Fmac.20180090</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>10.1257/mac.20180090</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Hansen, S., McMahon, M., &amp; Tong, M. (2019). The Long-Run Information Effect of Central Bank Communication. Journal of Monetary Economics, 108, 185-202.</t>
-        </is>
-      </c>
-      <c r="C12" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>https://ideas.repec.org/a/eee/moneco/v108y2019icp185-202.html</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>10.1016/j.jmoneco.2019.08.002</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Altavilla, C., Brugnolini, L., Gurkaynak, R. S., Motto, R., &amp; Ragusa, G. (2019). Measuring Euro Area Monetary Policy. Journal of Monetary Economics, 108, 162-179.</t>
-        </is>
-      </c>
-      <c r="C13" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>https://ideas.repec.org/a/eee/moneco/v108y2019icp162-179.html</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>10.1016/j.jmoneco.2019.08.016</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[8]</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>中国人民银行：《货币政策执行报告》，2006年第1季度至2026年第1季度，公开发布文本。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor monetary policy analysis and reporting
- Updated the stock volatility analysis to disable legacy ARX mean diagnostic and return a status note.
- Enhanced notebook execution to clear outputs and handle kernel configuration for better reproducibility.
- Added calculations for guidance novelty standard deviation and its effect on stock volatility to the paper builder.
- Revised references in the paper to include additional studies on central bank communication and monetary policy.
- Improved text clarity in the paper by refining sentences related to model diagnostics and validation processes.
</commit_message>
<xml_diff>
--- a/paper/引用一致性审计.xlsx
+++ b/paper/引用一致性审计.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,6 +553,96 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>[9]</t>
+        </is>
+      </c>
+      <c r="B10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>McMahon M., Schipke A. and Li X. China's Monetary Policy Communication: Frameworks, Impact, and Recommendations. IMF Working Paper, 2018/244.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Blinder A. S., Ehrmann M., Fratzscher M., de Haan J. and Jansen D. Central Bank Communication and Monetary Policy: A Survey of Theory and Evidence. Journal of Economic Literature, 2008, 46(4): 910-945.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[11]</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hansen S. and McMahon M. Shocking Language: Understanding the Macroeconomic Effects of Central Bank Communication. Journal of International Economics, 2016, 99: S114-S133.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>[12]</t>
+        </is>
+      </c>
+      <c r="B13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Nakamura E. and Steinsson J. High-Frequency Identification of Monetary Non-Neutrality: The Information Effect. Quarterly Journal of Economics, 2018, 133(3): 1283-1330.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[13]</t>
+        </is>
+      </c>
+      <c r="B14" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Jarocinski M. and Karadi P. Deconstructing Monetary Policy Surprises: The Role of Information Shocks. American Economic Journal: Macroeconomics, 2020, 12(2): 1-43.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[14]</t>
+        </is>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Kuttner K. N. Monetary Policy Surprises and Interest Rates: Evidence from the Fed Funds Futures Market. Journal of Monetary Economics, 2001, 47(3): 523-544.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add journal_style and journal_tables modules for reporting
- Implemented journal_style.py to define styles for document formatting, including page, font, paragraph, heading, table, figure, caption, header, footer, and reference styles.
- Added utility functions for setting font, paragraph formatting, section configuration, and table management.
- Created journal_tables.py to manage the generation of various tables related to monetary policy reports, including data formatting and writing to CSV and Excel files.
- Introduced data classes and helper functions for building structured tables from processed data.
</commit_message>
<xml_diff>
--- a/paper/引用一致性审计.xlsx
+++ b/paper/引用一致性审计.xlsx
@@ -413,234 +413,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>citation</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>appears_in_body</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>reference</t>
+          <t>body_author_year_cited</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>[1]</t>
+          <t>[1] 董青马，张皓越，马剑文，等．央行沟通与资产价格：识别“潜在”未预期货币政策信息[J]．金融研究，2024(6)．</t>
         </is>
       </c>
       <c r="B2" t="b">
         <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>姜富伟、胡逸驰、黄楠：《央行货币政策报告文本信息、宏观经济与股票市场》，《金融研究》，2021年第6期。</t>
-        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>[2]</t>
+          <t>[2] 姜富伟，胡逸驰，黄楠．央行货币政策报告文本信息、宏观经济与股票市场[J]．金融研究，2021(6)．</t>
         </is>
       </c>
       <c r="B3" t="b">
         <v>1</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>董青马、张皓越、马剑文、尚玉皇：《央行沟通与资产价格：识别“潜在”未预期货币政策信息》，《金融研究》，2024年第6期。</t>
-        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>[3]</t>
+          <t>[3] 尚玉皇，刘华，申峰．预期的博弈：央行沟通与国债收益率曲线[J]．金融研究，2025(9)．</t>
         </is>
       </c>
       <c r="B4" t="b">
         <v>1</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>尚玉皇、刘华、申峰：《预期的博弈：央行沟通与国债收益率曲线》，《金融研究》，2025年第9期。</t>
-        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[4] 中国人民银行．中国货币政策执行报告[R/OL]．2006-2025．</t>
         </is>
       </c>
       <c r="B5" t="b">
         <v>1</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Du Z., Huang A. G., Wermers R. and Wu W. Language and Domain Specificity: A Chinese Financial Sentiment Dictionary. Review of Finance, 2022, 26(3): 673-719.</t>
-        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>[5]</t>
+          <t>[5] Blinder A S, Ehrmann M, Fratzscher M, et al. Central Bank Communication and Monetary Policy: A Survey of Theory and Evidence[J]. Journal of Economic Literature, 2008, 46(4): 910-945.</t>
         </is>
       </c>
       <c r="B6" t="b">
         <v>1</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Gurkaynak R. S., Sack B. and Swanson E. Do Actions Speak Louder Than Words? The Response of Asset Prices to Monetary Policy Actions and Statements. International Journal of Central Banking, 2005, 1(1): 55-93.</t>
-        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>[6]</t>
+          <t>[6] Du Z, Huang A G, Wermers R, et al. Language and Domain Specificity: A Chinese Financial Sentiment Dictionary[J]. Review of Finance, 2022, 26(3): 673-719.</t>
         </is>
       </c>
       <c r="B7" t="b">
         <v>1</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Tetlock P. C. Giving Content to Investor Sentiment: The Role of Media in the Stock Market. Journal of Finance, 2007, 62(3): 1139-1168.</t>
-        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>[7]</t>
+          <t>[7] Ehrmann M, Talmi J. Starting from a Blank Page? Semantic Similarity in Central Bank Communication and Market Volatility[J]. Journal of Monetary Economics, 2020, 111: 48-62.</t>
         </is>
       </c>
       <c r="B8" t="b">
         <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Nelson D. B. Conditional Heteroskedasticity in Asset Returns: A New Approach. Econometrica, 1991, 59(2): 347-370.</t>
-        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>[8]</t>
+          <t>[8] Gurkaynak R S, Sack B, Swanson E T. Do Actions Speak Louder than Words? The Response of Asset Prices to Monetary Policy Actions and Statements[J]. International Journal of Central Banking, 2005, 1(1): 55-93.</t>
         </is>
       </c>
       <c r="B9" t="b">
         <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>中国人民银行：《货币政策执行报告》，2006年第1季度至2026年第1季度，公开发布文本。</t>
-        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>[9]</t>
+          <t>[9] Hansen S, McMahon M. Shocking Language: Understanding the Macroeconomic Effects of Central Bank Communication[J]. Journal of International Economics, 2016, 99(S1): S114-S133.</t>
         </is>
       </c>
       <c r="B10" t="b">
         <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>McMahon M., Schipke A. and Li X. China's Monetary Policy Communication: Frameworks, Impact, and Recommendations. IMF Working Paper, 2018/244.</t>
-        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>[10]</t>
+          <t>[10] Jarocinski M, Karadi P. Deconstructing Monetary Policy Surprises: The Role of Information Shocks[J]. American Economic Journal: Macroeconomics, 2020, 12(2): 1-43.</t>
         </is>
       </c>
       <c r="B11" t="b">
         <v>1</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Blinder A. S., Ehrmann M., Fratzscher M., de Haan J. and Jansen D. Central Bank Communication and Monetary Policy: A Survey of Theory and Evidence. Journal of Economic Literature, 2008, 46(4): 910-945.</t>
-        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>[11]</t>
+          <t>[11] Kuttner K N. Monetary Policy Surprises and Interest Rates: Evidence from the Fed Funds Futures Market[J]. Journal of Monetary Economics, 2001, 47(3): 523-544.</t>
         </is>
       </c>
       <c r="B12" t="b">
         <v>1</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Hansen S. and McMahon M. Shocking Language: Understanding the Macroeconomic Effects of Central Bank Communication. Journal of International Economics, 2016, 99: S114-S133.</t>
-        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[12] McMahon M, Schipke A, Li X. China's Monetary Policy Communication: Frameworks, Impact, and Recommendations[R]. IMF Working Paper, WP/18/244, 2018.</t>
         </is>
       </c>
       <c r="B13" t="b">
         <v>1</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Nakamura E. and Steinsson J. High-Frequency Identification of Monetary Non-Neutrality: The Information Effect. Quarterly Journal of Economics, 2018, 133(3): 1283-1330.</t>
-        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>[13]</t>
+          <t>[13] Nakamura E, Steinsson J. High-Frequency Identification of Monetary Non-Neutrality: The Information Effect[J]. Quarterly Journal of Economics, 2018, 133(3): 1283-1330.</t>
         </is>
       </c>
       <c r="B14" t="b">
         <v>1</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Jarocinski M. and Karadi P. Deconstructing Monetary Policy Surprises: The Role of Information Shocks. American Economic Journal: Macroeconomics, 2020, 12(2): 1-43.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>[14]</t>
-        </is>
-      </c>
-      <c r="B15" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Kuttner K. N. Monetary Policy Surprises and Interest Rates: Evidence from the Fed Funds Futures Market. Journal of Monetary Economics, 2001, 47(3): 523-544.</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>